<commit_message>
Dossier investisseur Halle v2 (logo, travaux du viaduc en juin-juillet, Gotham Light, version néerlandaise à la suite, feuille Food cost P&L) ; liste des produits de Halle avec leur coefficient (PDF + Excel) ; coefficients : recettes à vérifier signalées, groupe hérité de la catégorie
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RJV3ij12SyJdTDnhHEsPhb
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-2026-10/Halle-chiffres-2026.xlsx
+++ b/docs/dossiers/halle-2026-10/Halle-chiffres-2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Assortiment (sept.)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Semaine type" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Qualité T3 2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Food cost P&amp;L" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,10 +24,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
-    <numFmt numFmtId="165" formatCode="0.0 %"/>
-    <numFmt numFmtId="166" formatCode="0.00 €"/>
+    <numFmt numFmtId="165" formatCode="0.00 €"/>
+    <numFmt numFmtId="166" formatCode="0.0 %"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,12 +36,24 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="008D1D2C"/>
-      <sz val="14"/>
+      <sz val="12"/>
     </font>
     <font>
+      <name val="Arial"/>
+      <color rgb="007A736A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,7 +69,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -66,37 +79,44 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00D8D1C8"/>
+        <color rgb="00E6E0D8"/>
       </bottom>
-    </border>
-    <border>
-      <top style="thin">
-        <color rgb="00221E1A"/>
-      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -480,6 +500,7 @@
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,14 +510,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sources : API du panel (ventes, P&amp;L quotidien agrégé par mois), cockpit (food cost mesuré sur les recettes vendues, budget). Résultat opérationnel = CA − matière − main-d’œuvre − frais généraux. Chiffres hors TVA, en euros.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
+          <t>Sources : API du panel (ventes, P&amp;L quotidien agrégé par mois), cockpit (food cost mesuré sur les recettes vendues, budget). Résultat opérationnel = CA − matière − main-d’œuvre − frais généraux. Chiffres hors TVA, en euros. Juin et juillet 2026 : travaux sur le viaduc de Halle, effet estimé − 20 % (information du réseau, pas une mesure).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Mois</t>
@@ -572,487 +593,500 @@
           <t>Résultat %</t>
         </is>
       </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Février (ouverture le 20)</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="7" t="n">
         <v>6506.85</v>
       </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" t="n">
+      <c r="F5" s="6" t="n">
         <v>612</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="8" t="n">
         <v>10.63</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="9" t="n">
         <v>0.405</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="7" t="n">
         <v>2635.27</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="J5" s="7" t="n">
         <v>300</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="9" t="n">
         <v>0.046</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="7" t="n">
         <v>17234.56</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="9" t="n">
         <v>2.649</v>
       </c>
-      <c r="N5" s="4" t="n">
+      <c r="N5" s="7" t="n">
         <v>-13662.98</v>
       </c>
-      <c r="O5" s="5" t="n">
+      <c r="O5" s="9" t="n">
         <v>-2.099784073706939</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Mars</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>48767.34</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="7" t="n">
         <v>62000</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="9" t="n">
         <v>0.78657</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="6" t="n">
         <v>4341</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="8" t="n">
         <v>11.23</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="9" t="n">
         <v>0.398</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="7" t="n">
         <v>19409.4</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J6" s="7" t="n">
         <v>6334</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="9" t="n">
         <v>0.13</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" s="7" t="n">
         <v>9359.52</v>
       </c>
-      <c r="M6" s="5" t="n">
+      <c r="M6" s="9" t="n">
         <v>0.192</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" s="7" t="n">
         <v>13664.42</v>
       </c>
-      <c r="O6" s="5" t="n">
+      <c r="O6" s="9" t="n">
         <v>0.2801961312632594</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Avril</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="7" t="n">
         <v>55831.57</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="7" t="n">
         <v>62000</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="9" t="n">
         <v>0.9005091935483871</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="6" t="n">
         <v>4486</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G7" s="8" t="n">
         <v>12.45</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="9" t="n">
         <v>0.391</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="7" t="n">
         <v>21830.14</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="J7" s="7" t="n">
         <v>5814.5</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="9" t="n">
         <v>0.104</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="L7" s="7" t="n">
         <v>9608.700000000001</v>
       </c>
-      <c r="M7" s="5" t="n">
+      <c r="M7" s="9" t="n">
         <v>0.172</v>
       </c>
-      <c r="N7" s="4" t="n">
+      <c r="N7" s="7" t="n">
         <v>18578.23</v>
       </c>
-      <c r="O7" s="5" t="n">
+      <c r="O7" s="9" t="n">
         <v>0.3327549270063514</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Mai</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="7" t="n">
         <v>60239.57</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="7" t="n">
         <v>62000</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="9" t="n">
         <v>0.9716059677419355</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="6" t="n">
         <v>4756</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="G8" s="8" t="n">
         <v>12.67</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="9" t="n">
         <v>0.3720000000000001</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="7" t="n">
         <v>22409.12</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="J8" s="7" t="n">
         <v>10080.5</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="9" t="n">
         <v>0.167</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="L8" s="7" t="n">
         <v>19533.72</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M8" s="9" t="n">
         <v>0.324</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="N8" s="7" t="n">
         <v>8216.23</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="O8" s="9" t="n">
         <v>0.1363925738513738</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Juin</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="7" t="n">
         <v>46947.83</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="7" t="n">
         <v>62000</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="9" t="n">
         <v>0.7572230645161291</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="6" t="n">
         <v>3811</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G9" s="8" t="n">
         <v>12.32</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="9" t="n">
         <v>0.363</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I9" s="7" t="n">
         <v>17042.06</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="J9" s="7" t="n">
         <v>8714</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K9" s="9" t="n">
         <v>0.186</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="L9" s="7" t="n">
         <v>10658.7</v>
       </c>
-      <c r="M9" s="5" t="n">
+      <c r="M9" s="9" t="n">
         <v>0.227</v>
       </c>
-      <c r="N9" s="4" t="n">
+      <c r="N9" s="7" t="n">
         <v>10533.07</v>
       </c>
-      <c r="O9" s="5" t="n">
+      <c r="O9" s="9" t="n">
         <v>0.2243569085088704</v>
       </c>
+      <c r="P9" s="10" t="inlineStr">
+        <is>
+          <t>Travaux sur le viaduc de Halle : effet estimé − 20 % ; sans eux, environ 58 685 €</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Juillet</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="7" t="n">
         <v>46236.55</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="7" t="n">
         <v>62000</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="9" t="n">
         <v>0.745750806451613</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="6" t="n">
         <v>3776</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="G10" s="8" t="n">
         <v>12.25</v>
       </c>
-      <c r="H10" s="5" t="n">
+      <c r="H10" s="9" t="n">
         <v>0.368</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="7" t="n">
         <v>17015.05</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="J10" s="7" t="n">
         <v>8110.75</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="9" t="n">
         <v>0.175</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="L10" s="7" t="n">
         <v>13042.63</v>
       </c>
-      <c r="M10" s="5" t="n">
+      <c r="M10" s="9" t="n">
         <v>0.282</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="N10" s="7" t="n">
         <v>8068.12</v>
       </c>
-      <c r="O10" s="5" t="n">
+      <c r="O10" s="9" t="n">
         <v>0.1744965833307199</v>
       </c>
+      <c r="P10" s="10" t="inlineStr">
+        <is>
+          <t>Travaux sur le viaduc de Halle : effet estimé − 20 % ; sans eux, environ 57 796 €</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Août</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="7" t="n">
         <v>52350.95</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" s="7" t="n">
         <v>61000</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="9" t="n">
         <v>0.8582122950819672</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="6" t="n">
         <v>4323</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="G11" s="8" t="n">
         <v>12.11</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="9" t="n">
         <v>0.364</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="I11" s="7" t="n">
         <v>19055.75</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="J11" s="7" t="n">
         <v>8167.75</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="K11" s="9" t="n">
         <v>0.156</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="L11" s="7" t="n">
         <v>13042.63</v>
       </c>
-      <c r="M11" s="5" t="n">
+      <c r="M11" s="9" t="n">
         <v>0.249</v>
       </c>
-      <c r="N11" s="4" t="n">
+      <c r="N11" s="7" t="n">
         <v>12084.82</v>
       </c>
-      <c r="O11" s="5" t="n">
+      <c r="O11" s="9" t="n">
         <v>0.2308424202426126</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Septembre</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="7" t="n">
         <v>50849.75</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="7" t="n">
         <v>61000</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="9" t="n">
         <v>0.8336024590163934</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="6" t="n">
         <v>4156</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="G12" s="8" t="n">
         <v>12.24</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="9" t="n">
         <v>0.362</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="I12" s="7" t="n">
         <v>18407.61</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="J12" s="7" t="n">
         <v>9477.5</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="K12" s="9" t="n">
         <v>0.186</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="L12" s="7" t="n">
         <v>13042.8</v>
       </c>
-      <c r="M12" s="5" t="n">
+      <c r="M12" s="9" t="n">
         <v>0.256</v>
       </c>
-      <c r="N12" s="4" t="n">
+      <c r="N12" s="7" t="n">
         <v>9921.84</v>
       </c>
-      <c r="O12" s="5" t="n">
+      <c r="O12" s="9" t="n">
         <v>0.1951207233073909</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Octobre (1 → 8)</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="7" t="n">
         <v>15628.2</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" s="7" t="n">
         <v>61000</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="9" t="n">
         <v>0.2562</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="6" t="n">
         <v>1313</v>
       </c>
-      <c r="G13" s="6" t="n">
+      <c r="G13" s="8" t="n">
         <v>11.9</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="9" t="n">
         <v>0.404</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" s="7" t="n">
         <v>6313.79</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="J13" s="7" t="n">
         <v>3502.75</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="K13" s="9" t="n">
         <v>0.224</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="L13" s="7" t="n">
         <v>4377.42</v>
       </c>
-      <c r="M13" s="5" t="n">
+      <c r="M13" s="9" t="n">
         <v>0.28</v>
       </c>
-      <c r="N13" s="4" t="n">
+      <c r="N13" s="7" t="n">
         <v>1434.24</v>
       </c>
-      <c r="O13" s="5" t="n">
+      <c r="O13" s="9" t="n">
         <v>0.09177256497869236</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Cumul mars → septembre (7 mois pleins)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="6" t="n">
         <v>213</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>361223.56</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="7" t="n">
         <v>432000</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>0.8361656481481481</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="6" t="n">
         <v>29649</v>
       </c>
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="8" t="n">
         <v>12.1833302978178</v>
       </c>
       <c r="H14" s="9" t="n">
         <v>0.3741979897435261</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="7" t="n">
         <v>135169.13</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="7" t="n">
         <v>56699</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0.1569637373597669</v>
       </c>
-      <c r="L14" s="8" t="n">
+      <c r="L14" s="7" t="n">
         <v>88288.7</v>
       </c>
       <c r="M14" s="9" t="n">
         <v>0.2444156743264476</v>
       </c>
-      <c r="N14" s="8" t="n">
+      <c r="N14" s="7" t="n">
         <v>81066.73</v>
       </c>
       <c r="O14" s="9" t="n">
@@ -1061,7 +1095,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1089,6 +1123,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1112,78 +1147,78 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Food cost (matière, % du CA)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="9" t="n">
         <v>0.3741979897435261</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="9" t="n">
         <v>0.3960000000000001</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="9" t="n">
         <v>0.32</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Main-d’œuvre (% du CA, telle qu’encodée au panel)</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="9" t="n">
         <v>0.1569637373597669</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="9" t="n">
         <v>0.1894908403962734</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="9" t="n">
         <v>0.33</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Frais généraux (% du CA, montant mensuel encodé au panel)</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.2444156743264476</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="9" t="n">
         <v>0.2825339620840834</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.135</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Panier moyen (€)</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="8" t="n">
         <v>12.1833302978178</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="8" t="n">
         <v>14.25714285714286</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Atteinte du budget CA</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.8361656481481481</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Les trois autres magasins : Corbais, Gosselies, Sombreffe. Un mois dont le food cost mesuré dépasse 60 % (anomalie de recette) est écarté de la moyenne.</t>
         </is>
@@ -1219,8 +1254,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Rythme actuel : CA mensuel moyen mars → septembre = 51 603 €. Ces postes sont ceux du modèle  pas des montants constatés : le loyer réel vient du bail.</t>
         </is>
@@ -1264,336 +1299,333 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Matière,première &amp; Emballage</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Matière première</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="9" t="n">
         <v>0.36</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Matière,première &amp; Emballage</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Emballage</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.02</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Loyer + charges locatives</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="9" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="7" t="n">
         <v>3612</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Fixe</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Selon emplacement</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Énergie (eau, gaz, électricité)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="9" t="n">
         <v>0.05</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="9" t="n">
         <v>0.05</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="7" t="n">
         <v>2580</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Groupement d’achat, appel d’offres</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Variable selon la saison</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Maintenance &amp; nettoyage</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="9" t="n">
         <v>0.01</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="9" t="n">
         <v>0.005</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="7" t="n">
         <v>516</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Préventif et régulier</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Entretien du matériel</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Assurances, licences, etc.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="9" t="n">
         <v>0.01</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="9" t="n">
         <v>0.01</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="7" t="n">
         <v>516</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Suivi des échéances</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Redevances de marque</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Royalties franchise</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="9" t="n">
         <v>0.02</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="9" t="n">
         <v>0.02</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="7" t="n">
         <v>1032</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Fixe</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Redevance marque</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Redevances de marque</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Redevance assistance</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="7" t="n">
         <v>774</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Fixe</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Accompagnement franchiseur</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Redevances de marque</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Marketing national / local</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="7" t="n">
         <v>774</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Fixe</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Investissement</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Amortissements / leasing matériel</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="9" t="n">
         <v>0.05</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="9" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="7" t="n">
         <v>2580</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Fixe</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>Machines, mobilier</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Frais généraux</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Autres (comptabilité, banque, divers)</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="9" t="n">
         <v>0.015</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="7" t="n">
         <v>774</v>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Optimisation des prestataires</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Total des postes budgétés</t>
         </is>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="9" t="n">
         <v>0.255</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="7" t="n">
         <v>13159</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1622,6 +1654,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1655,645 +1688,645 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Viennoiserie Ind.</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Viennoiserie</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="7" t="n">
         <v>14551.9</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="9" t="n">
         <v>0.286174464967871</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="6" t="n">
         <v>7564</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="7" t="n">
         <v>8032.9</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="9" t="n">
         <v>0.1579732447062178</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="6" t="n">
         <v>741</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="6" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Pain</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Boulangerie</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>6244.6</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.122804930211063</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="6" t="n">
         <v>2045</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Petite Boulangerie</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Boulangerie</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="7" t="n">
         <v>4590.8</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.09028166313502033</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7" s="6" t="n">
         <v>4096</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Quiches</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Quiches</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="7" t="n">
         <v>3463.9</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="9" t="n">
         <v>0.06812029557667441</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="6" t="n">
         <v>391</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="6" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Sandwiches garnis</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Traiteur</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="7" t="n">
         <v>1985.55</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="9" t="n">
         <v>0.03904738961351826</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9" s="6" t="n">
         <v>344</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="6" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Cookies</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Biscuiterie</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="7" t="n">
         <v>1460.1</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="9" t="n">
         <v>0.02871400547691975</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10" s="6" t="n">
         <v>573</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Tartissières - 19Ø</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="7" t="n">
         <v>1225.1</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="9" t="n">
         <v>0.02409254716099882</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="6" t="n">
         <v>69</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Entremets - 190Ø</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="7" t="n">
         <v>979.9</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="9" t="n">
         <v>0.01927049788838687</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Boissons froides</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Boissons</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="7" t="n">
         <v>922.1</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="9" t="n">
         <v>0.018133815800471</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="6" t="n">
         <v>345</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="6" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Viennoiserie réduction</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Viennoiserie</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="7" t="n">
         <v>858.6</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="9" t="n">
         <v>0.01688503876616896</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14" s="6" t="n">
         <v>869</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Tartissières - 12Ø</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="7" t="n">
         <v>841.5</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="9" t="n">
         <v>0.01654875392701046</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie individuelle</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="7" t="n">
         <v>747</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="9" t="n">
         <v>0.01469033771060821</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="6" t="n">
         <v>249</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Pain Tradition</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Boulangerie</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="7" t="n">
         <v>643.3</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="9" t="n">
         <v>0.01265099631758268</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="6" t="n">
         <v>174</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="6" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Épicerie</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Épicerie</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="7" t="n">
         <v>633.6</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="9" t="n">
         <v>0.01246023825092552</v>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Cake</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="7" t="n">
         <v>616</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="9" t="n">
         <v>0.01211412052173315</v>
       </c>
-      <c r="E19" t="n">
+      <c r="E19" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="6" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Entremets - Individuel</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="7" t="n">
         <v>574.1</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="9" t="n">
         <v>0.01129012433689448</v>
       </c>
-      <c r="E20" t="n">
+      <c r="E20" s="6" t="n">
         <v>185</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Entremets - 4/6 personnes</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Pâtisserie · Tartes</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="7" t="n">
         <v>566.2</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="9" t="n">
         <v>0.01113476467435926</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Croutes Fruits Frais</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="7" t="n">
         <v>405</v>
       </c>
-      <c r="D22" s="5" t="n">
+      <c r="D22" s="9" t="n">
         <v>0.007964640927438187</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E22" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="F22" t="n">
+      <c r="F22" s="6" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Boissons chaudes</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Boissons</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="7" t="n">
         <v>284.7</v>
       </c>
-      <c r="D23" s="5" t="n">
+      <c r="D23" s="9" t="n">
         <v>0.00559884758528803</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="6" t="n">
         <v>114</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F23" s="6" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Tarte Fruits Frais</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="7" t="n">
         <v>278.8</v>
       </c>
-      <c r="D24" s="5" t="n">
+      <c r="D24" s="9" t="n">
         <v>0.005482819482888313</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E24" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Tartes – Ø 28 cm</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="7" t="n">
         <v>278.6</v>
       </c>
-      <c r="D25" s="5" t="n">
+      <c r="D25" s="9" t="n">
         <v>0.005478886326874764</v>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F25" t="n">
+      <c r="F25" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Tartes au sucre</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Tartes</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="7" t="n">
         <v>222.6</v>
       </c>
-      <c r="D26" s="5" t="n">
+      <c r="D26" s="9" t="n">
         <v>0.004377602643080841</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="F26" t="n">
+      <c r="F26" s="6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Wrapps</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Traiteur</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="7" t="n">
         <v>208</v>
       </c>
-      <c r="D27" s="5" t="n">
+      <c r="D27" s="9" t="n">
         <v>0.004090482254091712</v>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="F27" t="n">
+      <c r="F27" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Glace by Rawette</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Épicerie</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="7" t="n">
         <v>132</v>
       </c>
-      <c r="D28" s="5" t="n">
+      <c r="D28" s="9" t="n">
         <v>0.002595882968942817</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="6" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Biscuiterie</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Biscuiterie</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="7" t="n">
         <v>102.9</v>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" s="9" t="n">
         <v>0.002023608768971332</v>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="6" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Sans catégorie</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="5" t="n">
+      <c r="D30" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="n">
+      <c r="E30" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2324,6 +2357,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2347,114 +2381,114 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>lundi</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="7" t="n">
         <v>1239.9</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="9" t="n">
         <v>0.106</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>mardi</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="7" t="n">
         <v>1271.79</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="9" t="n">
         <v>0.109</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>mercredi</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>1339.02</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="9" t="n">
         <v>0.111</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>jeudi</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="7" t="n">
         <v>1221.37</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="9" t="n">
         <v>0.101</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>vendredi</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="7" t="n">
         <v>1491.06</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="9" t="n">
         <v>0.124</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>samedi</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="7" t="n">
         <v>2492.35</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="9" t="n">
         <v>0.207</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>dimanche</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="7" t="n">
         <v>2807.97</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="9" t="n">
         <v>0.241</v>
       </c>
     </row>
@@ -2484,6 +2518,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -2502,83 +2537,83 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Note Google</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="6" t="n">
         <v>4.5</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>46 avis, relevé du 2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Client mystère</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>75 / 100</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>note reçue au trimestre</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Tâches rendues</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>34 %</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>586 rendues sur 1742 attendues, 92 jours</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Atteinte du budget</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>81.2 %</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>CA 149 440 € sur un budget de 184 000 €</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>12.09 / 20</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>rang 2 sur 4 magasins, 3.02 étoiles sur 5</t>
         </is>
@@ -2587,4 +2622,555 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Le food cost lu dans le P&amp;L du cockpit (recettes vendues, ticket par ticket) — Halle et réseau</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Depuis le 1er août 2026, le cockpit lit chaque ticket et recompose le coût matière des recettes vendues au coût de recette du jour. Avant août, les tickets ne sont pas lus : le dossier utilise la marge mesurée par le panel (feuille Mois par mois). Les deux mesures diffèrent : voir la colonne de comparaison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Période</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Du</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>CA Halle</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Matière Halle (P&amp;L)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Food cost Halle (P&amp;L)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Food cost réseau (P&amp;L)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Food cost Halle (panel, dossier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-03</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>48767.34</v>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>tickets non lus</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0.398</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-04</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>55831.57</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>tickets non lus</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0.391</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-05</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>60278.02</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>tickets non lus</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>0.3720000000000001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-06</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>46950.55</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>tickets non lus</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>0.363</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-07</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>46239.03</v>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>tickets non lus</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>0.368</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-08</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>52350.95</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>23219.97</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>0.444</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>0.364</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-09</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>50849.75</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>22096.21</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0.413</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0.362</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Mois 2026-10</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>15707.4</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>6323.39</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>0.403</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.399</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0.404</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-08-17</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>12400.55</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>5456.53</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>0.418</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-08-24</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>11320.2</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>5034.96</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0.418</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-08-31</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>11530.15</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>5083.85</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>0.417</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-09-07</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>12077.9</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>5257.52</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>0.435</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0.414</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-09-14</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>12591.7</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>5425.58</v>
+      </c>
+      <c r="F17" s="9" t="n">
+        <v>0.431</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0.409</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-09-21</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>11908.45</v>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>5144.82</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>0.4320000000000001</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>0.408</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-09-28</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>12864.2</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>5404.51</v>
+      </c>
+      <c r="F19" s="9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>0.413</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Semaine du 2026-10-05</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>6785.65</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>2651.9</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>0.391</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Dossier investisseur Halle v3 : marges par catégorie et poids dans le chiffre (septembre), page des outils de gestion avec les écrans du dashboard de Halle ; feuille Excel des marges
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RJV3ij12SyJdTDnhHEsPhb
</commit_message>
<xml_diff>
--- a/docs/dossiers/halle-2026-10/Halle-chiffres-2026.xlsx
+++ b/docs/dossiers/halle-2026-10/Halle-chiffres-2026.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Semaine type" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Qualité T3 2026" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Food cost P&amp;L" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Marges par catégorie" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,10 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
     <numFmt numFmtId="165" formatCode="0.00 €"/>
     <numFmt numFmtId="166" formatCode="0.0 %"/>
+    <numFmt numFmtId="167" formatCode="× 0.00"/>
+    <numFmt numFmtId="168" formatCode="0 %"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -86,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
@@ -116,6 +119,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3173,4 +3182,1039 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Les marges par catégorie et leur poids dans le chiffre — septembre 2026, Halle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Marge brute = chiffre − coût de recette, telle que le panel la chiffre produit par produit ; les recettes invraisemblables (coût au-dessus du prix ou sous 5 % de celui-ci) sont écartées. « Coût connu » : la part du chiffre de la catégorie dont le coût est mesuré.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Part du CA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Pièces</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Références</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Food cost</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Marge brute</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Coefficient</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Coût connu (part du CA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Viennoiserie Ind.</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Viennoiserie</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0.286174464967871</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>14551.9</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>7564</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>0.4222012245823569</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0.577798775417643</v>
+      </c>
+      <c r="I5" s="12" t="n">
+        <v>2.368538843034394</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0.1579732447062178</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <v>8032.9</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>741</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>0.3874197124071851</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0.6125802875928148</v>
+      </c>
+      <c r="I6" s="12" t="n">
+        <v>2.581179965744701</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>0.819840904281144</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Pain</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Boulangerie</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>0.122804930211063</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>6244.6</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>2045</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>0.5735979886622042</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>0.4264020113377958</v>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>1.74338128753256</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Petite Boulangerie</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Boulangerie</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>0.09028166313502034</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>4590.8</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>4096</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>0.4612551189335191</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>0.5387448810664809</v>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>2.167997619868432</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Quiches</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Quiches</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0.06812029557667441</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>3463.9</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>391</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>0.2742902521342069</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>0.7257097478657931</v>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>3.645773016792125</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>0.1454141285833886</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Sandwiches garnis</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Traiteur</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>0.03904738961351826</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>1985.55</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>344</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>0.4123153970918819</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>0.5876846029081182</v>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>2.425327812284333</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>0.8849689003047015</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Cookies</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Biscuiterie</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0.02871400547691975</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1460.1</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>0.3749537702897062</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0.6250462297102939</v>
+      </c>
+      <c r="I11" s="12" t="n">
+        <v>2.666995451805579</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Tartissières - 19Ø</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>0.02409254716099882</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1225.1</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>0.4758305444453515</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>0.5241694555546486</v>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>2.101588499674066</v>
+      </c>
+      <c r="J12" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Entremets - 190Ø</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>0.01927049788838687</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>979.9</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Boissons froides</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Boissons</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0.018133815800471</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>922.1</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>345</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>0.355174314455009</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>0.644825685544991</v>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>2.815518913676042</v>
+      </c>
+      <c r="J14" s="13" t="n">
+        <v>0.7870079167118534</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Viennoiserie réduction</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Viennoiserie</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>0.01688503876616896</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>858.6</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>869</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>0.4841719077568135</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>0.5158280922431866</v>
+      </c>
+      <c r="I15" s="12" t="n">
+        <v>2.065382117341416</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Tartissières - 12Ø</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>0.01654875392701046</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>841.5</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>0.4432722284574136</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>0.5567277715425863</v>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>2.255950036572329</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0.9529411764705884</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie individuelle</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>0.01469033771060821</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>747</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>249</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I17" s="12" t="n">
+        <v>5.555555555555555</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Pain Tradition</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Boulangerie</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>0.01265099631758268</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>643.3</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>174</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>0.4810041971086585</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>0.5189958028913415</v>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>2.078983938208965</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Épicerie</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Épicerie</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>0.01246023825092552</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>633.6</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>0.3697175840032982</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>0.6302824159967018</v>
+      </c>
+      <c r="I19" s="12" t="n">
+        <v>2.704767214942849</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>0.765625</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Cake</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>0.01211412052173315</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>616</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>0.442435064935065</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>0.557564935064935</v>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>2.260218683496</v>
+      </c>
+      <c r="J20" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Entremets - Individuel</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>0.01129012433689448</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>574.1</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>185</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>0.3850766456266908</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>0.6149233543733092</v>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>2.59688561058424</v>
+      </c>
+      <c r="J21" s="13" t="n">
+        <v>0.772687685072287</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Entremets - 4/6 personnes</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Pâtisserie · Tartes</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>0.01113476467435926</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>566.2</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Croutes Fruits Frais</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>0.007964640927438187</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>405</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Boissons chaudes</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Boissons</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="n">
+        <v>0.00559884758528803</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>284.7</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>0.06956521739130435</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>0.9304347826086956</v>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>14.375</v>
+      </c>
+      <c r="J24" s="13" t="n">
+        <v>0.5089567966280295</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Tarte Fruits Frais</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="n">
+        <v>0.005482819482888313</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>278.8</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>0.2805595408895265</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>0.7194404591104735</v>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>3.564305804142163</v>
+      </c>
+      <c r="J25" s="13" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Tartes – Ø 28 cm</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="n">
+        <v>0.005478886326874765</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>278.6</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>0.5005025125628141</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>0.499497487437186</v>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>1.997991967871486</v>
+      </c>
+      <c r="J26" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Tartes au sucre</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Tartes</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="n">
+        <v>0.004377602643080842</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>222.6</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>0.2987421383647799</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>0.7012578616352201</v>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>3.347368421052632</v>
+      </c>
+      <c r="J27" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Wrapps</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Traiteur</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="n">
+        <v>0.004090482254091712</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>208</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>0.2495673076923077</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>0.7504326923076923</v>
+      </c>
+      <c r="I28" s="12" t="n">
+        <v>4.006935079946061</v>
+      </c>
+      <c r="J28" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Glace by Rawette</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Épicerie</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n">
+        <v>0.002595882968942817</v>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>132</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>0.5359848484848486</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>0.4640151515151514</v>
+      </c>
+      <c r="I29" s="12" t="n">
+        <v>1.865724381625441</v>
+      </c>
+      <c r="J29" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Biscuiterie</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Biscuiterie</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="n">
+        <v>0.002023608768971332</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>0.4448979591836734</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>0.5551020408163265</v>
+      </c>
+      <c r="I30" s="12" t="n">
+        <v>2.247706422018349</v>
+      </c>
+      <c r="J30" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Toutes catégories</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>50849.75</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>18201</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>163</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>0.4344599219639492</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>0.5655400780360508</v>
+      </c>
+      <c r="I31" s="12" t="n">
+        <v>2.301708280661567</v>
+      </c>
+      <c r="J31" s="13" t="n">
+        <v>0.8575863204833848</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>